<commit_message>
Added New Configs and Improved Previous
</commit_message>
<xml_diff>
--- a/input/products.xlsx
+++ b/input/products.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="11">
   <si>
     <t>url</t>
   </si>
@@ -28,7 +28,7 @@
     <t>error</t>
   </si>
   <si>
-    <t>https://www.tatacliq.com/renee-natural-makeup-fixer-75-ml/p-mp000000027720317</t>
+    <t>https://www.vijaysales.com/p/191494/ifb-20-ltrs-convection-microwave-20pm-mec2-white</t>
   </si>
   <si>
     <t/>
@@ -37,16 +37,13 @@
     <t>done</t>
   </si>
   <si>
-    <t>2026-09-17T09:31:01.769Z</t>
-  </si>
-  <si>
-    <t>https://www.tatacliq.com/pac-micro-finish-makeup-fixer-120-ml/p-mp000000015561989</t>
-  </si>
-  <si>
-    <t>https://www.tatacliq.com/lakme-makeup-skincare-vit-c-superglow-skin-perfecting-makeup-fixer-60-ml/p-mp000000022501402</t>
-  </si>
-  <si>
-    <t>https://www.tatacliq.com/daily-life-forever52-all-day-long-makeup-fixer-100-ml/p-mp000000025883622</t>
+    <t>2026-09-18T05:37:04.759Z</t>
+  </si>
+  <si>
+    <t>https://www.vijaysales.com/p/109229/lg-20-ltrs-solo-microwave-ms2043db-black</t>
+  </si>
+  <si>
+    <t>https://www.vijaysales.com/p/224298/morphy-richards-29-litres-rcad-digi-oven-toaster-griller-with-13-preset-menu-digital-display-ai-preset-menu-knob-control-deep-blue</t>
   </si>
 </sst>
 </file>
@@ -423,7 +420,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -490,20 +487,6 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" t="s">
-        <v>8</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
SO Good Updates & Myntra Config
</commit_message>
<xml_diff>
--- a/input/products.xlsx
+++ b/input/products.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="60">
   <si>
     <t>url</t>
   </si>
@@ -28,7 +28,7 @@
     <t>error</t>
   </si>
   <si>
-    <t>https://www.vijaysales.com/p/191494/ifb-20-ltrs-convection-microwave-20pm-mec2-white</t>
+    <t>https://www.myntra.com/tshirts/wrogn/wrogn-pure-cotton-striped-polo-collar-slim-fit-t-shirt/26531622/buy</t>
   </si>
   <si>
     <t/>
@@ -37,13 +37,160 @@
     <t>done</t>
   </si>
   <si>
-    <t>2026-09-18T05:37:04.759Z</t>
-  </si>
-  <si>
-    <t>https://www.vijaysales.com/p/109229/lg-20-ltrs-solo-microwave-ms2043db-black</t>
-  </si>
-  <si>
-    <t>https://www.vijaysales.com/p/224298/morphy-richards-29-litres-rcad-digi-oven-toaster-griller-with-13-preset-menu-digital-display-ai-preset-menu-knob-control-deep-blue</t>
+    <t>2026-09-25T04:00:44.965Z</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/french+connection/french-connection-men-striped-polo-collar-pure-cotton-t-shirt/21388860/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/levis/levis-men-soft-pure-cotton-round-neck-half-sleeve-tshirt/12027436/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/levis/levis-men-soft-pure-cotton-round-neck-half-sleeve-tshirt/12027432/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/adidas/adidas-men-printed-pure-cotton-t-shirt/34149996/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/pepe+jeans/pepe-jeans-men-crew-neck-relaxed-fit-lounge-tshirt/33353185/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/roadsail/roadsail-men-scuderia-ferrari-formula-1-printed-drop-shoulder-sleeves-t-shirt/45728425/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/prosharx/prosharx-men-colourblocked-compression-t-shirt/44993306/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/levis/levis-men-soft-pure-cotton-round-neck-half-sleeve-tshirt/12027422/buy</t>
+  </si>
+  <si>
+    <t>2026-09-25T04:00:44.966Z</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/u.s.+polo+assn./us-polo-assn-men-embroidered-logo-pure-cotton-lightweight-lounge-t-shirt/22492582/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/bene+kleed/bene-kleed-men-regular-fit-embroidered-t-shirt/41737229/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/oishee/oishee-unisex-striped-t-shirt/46425378/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/here%26now/herenow-men-colourblocked-polo-collar-t-shirt/46222266/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/hrx+by+hrithik+roshan/hrx-by-hrithik-roshan-men-printed-running-rapid-dry-t-shirt/29010960/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/damensch/damensch-ultralight-basic-crew-pure-cotton-lounge-t-shirts/30205303/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/levis/levis-men-soft-pure-cotton-round-neck-half-sleeve-tshirt/12027418/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/kook+n+keech/kook-n-keech-drop-shoulder-sleeves-oversized-pure-cotton-t-shirt/27506790/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/xyxx/xyxx-men-pace-intellieaze-cotton-t-shirt/24026378/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/hrx+by+hrithik+roshan/hrx-by-hrithik-roshan-men-colourblocked-t-shirt/44709936/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/prosharx/prosharx-men-brand-logo-dri-fit-compression-t-shirt/44591460/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/cahoot/cahoot-men-solid-polo-collar-cotton-t-shirt/32193183/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/pepe+jeans/pepe-jeans-men-crew-neck-relaxed-fit-lounge-tshirt/32762106/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/imsa+moda/imsa-moda-men-colourblocked-t-shirt/46258981/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/van+heusen+innerwear/van-heusen-men-cotton-crew-neck-solid-regular-fit-short-sleeves-lounge-tshirt/30104756/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/the+modvue/the-modvue-men-brand-logo-dyed-t-shirt/45812329/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/the+indian+garage+co/the-indian-garage-co-men-t-shirt/40199466/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/damensch/damensch-ultralight-basic-crew-pure-cotton-lounge-t-shirts/30205304/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/cahoot/cahoot-men-self-design-polo-collar-cotton-t-shirt/32193190/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/prosharx/prosharx-men-brand-logo-dri-fit-compression-t-shirt/41918326/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/u.s.+polo+assn./us-polo-assn-men-pure-cotton-comfort-fit-lounge-t-shirt/36468833/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/v-mart/v-mart-men-polo-collar-slim-fit-t-shirt/46155716/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/hrx+by+hrithik+roshan/hrx-by-hrithik-roshan-men-brand-logo-printed-t-shirt/41509398/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/van+heusen+innerwear/van-heusen-innerwear-cotton-crew-neck-regular-short-sleeves-soft-breathable-lounge-tshirt/29638056/buy</t>
+  </si>
+  <si>
+    <t>2026-09-25T04:00:44.967Z</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/damensch/damensch-neo-cool-pure-cotton-regular-fit-tank-lounge-t-shirt/19563322/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/glitchez/glitchez-printed-oversized-fit-t-shirt/31819294/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/cahoot/cahoot-men-self-design-polo-collar-cotton-t-shirt/32193132/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/hotfits/hotfits-men-typography-printed-organic-cotton-t-shirt/46315858/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts-smart/urban+trees/urban-trees-printed-cotton-round-neck-tshirts/42543341/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/pepe+jeans/pepe-jeans-men-crew-neck-relaxed-fit-lounge-tshirt/32762104/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/damensch/damensch-men-ultralight-basic-crew-pure-cotton-lounge-t-shirts/30205305/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/gap/gap-brand-logo-printed-pure-cotton-slim-fit-t-shirt/40934832/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/pepe+jeans/pepe-jeans-round-neck-cotton-t-shirt/34851621/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/teevybe/teevybe-men-typography-printed-t-shirt/46330752/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/adidas/adidas-3-stripes-pure-cotton-t-shirt/35840598/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/lounge-tshirts/van+heusen+innerwear/van-heusen-innerwear-cotton-crew-neck-solid--short-sleeves-soft-breathable-lounge-tshirts/29638088/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/bdsquare/bdsquare-men-drop-shoulder-sleeves-t-shirt/39825768/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/nostrum/nostrum-men-solid-polo-collar-regular-fit-half-sleeve-t-shirt/33617040/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/flying+machine/flying-machine-pure-cotton-relaxed-fit-t-shirt/31598705/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/roadster/roadster-men-ready-to-wear-short-sleeves-typography-printed-t-shirt/46383516/buy</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/tshirts/mast+%26+harbour/mast--harbour-men-oversized-printed-t-shirt/45606383/buy</t>
   </si>
 </sst>
 </file>
@@ -420,7 +567,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -487,6 +634,664 @@
         <v>8</v>
       </c>
     </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" t="s">
+        <v>7</v>
+      </c>
+      <c r="D16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" t="s">
+        <v>7</v>
+      </c>
+      <c r="D21" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>36</v>
+      </c>
+      <c r="B29" t="s">
+        <v>6</v>
+      </c>
+      <c r="C29" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>37</v>
+      </c>
+      <c r="B30" t="s">
+        <v>6</v>
+      </c>
+      <c r="C30" t="s">
+        <v>7</v>
+      </c>
+      <c r="D30" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>38</v>
+      </c>
+      <c r="B31" t="s">
+        <v>6</v>
+      </c>
+      <c r="C31" t="s">
+        <v>7</v>
+      </c>
+      <c r="D31" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33" t="s">
+        <v>6</v>
+      </c>
+      <c r="C33" t="s">
+        <v>7</v>
+      </c>
+      <c r="D33" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>41</v>
+      </c>
+      <c r="B34" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>43</v>
+      </c>
+      <c r="B35" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>44</v>
+      </c>
+      <c r="B36" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>45</v>
+      </c>
+      <c r="B37" t="s">
+        <v>6</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>46</v>
+      </c>
+      <c r="B38" t="s">
+        <v>6</v>
+      </c>
+      <c r="C38" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>47</v>
+      </c>
+      <c r="B39" t="s">
+        <v>6</v>
+      </c>
+      <c r="C39" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>48</v>
+      </c>
+      <c r="B40" t="s">
+        <v>6</v>
+      </c>
+      <c r="C40" t="s">
+        <v>7</v>
+      </c>
+      <c r="D40" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>49</v>
+      </c>
+      <c r="B41" t="s">
+        <v>6</v>
+      </c>
+      <c r="C41" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>50</v>
+      </c>
+      <c r="B42" t="s">
+        <v>6</v>
+      </c>
+      <c r="C42" t="s">
+        <v>7</v>
+      </c>
+      <c r="D42" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>51</v>
+      </c>
+      <c r="B43" t="s">
+        <v>6</v>
+      </c>
+      <c r="C43" t="s">
+        <v>7</v>
+      </c>
+      <c r="D43" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>52</v>
+      </c>
+      <c r="B44" t="s">
+        <v>6</v>
+      </c>
+      <c r="C44" t="s">
+        <v>7</v>
+      </c>
+      <c r="D44" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>53</v>
+      </c>
+      <c r="B45" t="s">
+        <v>6</v>
+      </c>
+      <c r="C45" t="s">
+        <v>7</v>
+      </c>
+      <c r="D45" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>54</v>
+      </c>
+      <c r="B46" t="s">
+        <v>6</v>
+      </c>
+      <c r="C46" t="s">
+        <v>7</v>
+      </c>
+      <c r="D46" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>55</v>
+      </c>
+      <c r="B47" t="s">
+        <v>6</v>
+      </c>
+      <c r="C47" t="s">
+        <v>7</v>
+      </c>
+      <c r="D47" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>56</v>
+      </c>
+      <c r="B48" t="s">
+        <v>6</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>57</v>
+      </c>
+      <c r="B49" t="s">
+        <v>6</v>
+      </c>
+      <c r="C49" t="s">
+        <v>7</v>
+      </c>
+      <c r="D49" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>58</v>
+      </c>
+      <c r="B50" t="s">
+        <v>6</v>
+      </c>
+      <c r="C50" t="s">
+        <v>7</v>
+      </c>
+      <c r="D50" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>59</v>
+      </c>
+      <c r="B51" t="s">
+        <v>6</v>
+      </c>
+      <c r="C51" t="s">
+        <v>7</v>
+      </c>
+      <c r="D51" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
Improved UI of the Desgin , New Over Card UI
</commit_message>
<xml_diff>
--- a/input/products.xlsx
+++ b/input/products.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="59">
   <si>
     <t>url</t>
   </si>
@@ -37,7 +37,7 @@
     <t>done</t>
   </si>
   <si>
-    <t>2026-09-25T04:00:44.965Z</t>
+    <t>2026-09-25T11:52:31.380Z</t>
   </si>
   <si>
     <t>https://www.myntra.com/tshirts/french+connection/french-connection-men-striped-polo-collar-pure-cotton-t-shirt/21388860/buy</t>
@@ -64,9 +64,6 @@
     <t>https://www.myntra.com/lounge-tshirts/levis/levis-men-soft-pure-cotton-round-neck-half-sleeve-tshirt/12027422/buy</t>
   </si>
   <si>
-    <t>2026-09-25T04:00:44.966Z</t>
-  </si>
-  <si>
     <t>https://www.myntra.com/lounge-tshirts/u.s.+polo+assn./us-polo-assn-men-embroidered-logo-pure-cotton-lightweight-lounge-t-shirt/22492582/buy</t>
   </si>
   <si>
@@ -139,10 +136,10 @@
     <t>https://www.myntra.com/lounge-tshirts/van+heusen+innerwear/van-heusen-innerwear-cotton-crew-neck-regular-short-sleeves-soft-breathable-lounge-tshirt/29638056/buy</t>
   </si>
   <si>
-    <t>2026-09-25T04:00:44.967Z</t>
-  </si>
-  <si>
     <t>https://www.myntra.com/lounge-tshirts/damensch/damensch-neo-cool-pure-cotton-regular-fit-tank-lounge-t-shirt/19563322/buy</t>
+  </si>
+  <si>
+    <t>2026-09-25T11:52:31.381Z</t>
   </si>
   <si>
     <t>https://www.myntra.com/tshirts/glitchez/glitchez-printed-oversized-fit-t-shirt/31819294/buy</t>
@@ -715,12 +712,12 @@
         <v>7</v>
       </c>
       <c r="D10" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B11" t="s">
         <v>6</v>
@@ -729,12 +726,12 @@
         <v>7</v>
       </c>
       <c r="D11" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B12" t="s">
         <v>6</v>
@@ -743,12 +740,12 @@
         <v>7</v>
       </c>
       <c r="D12" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B13" t="s">
         <v>6</v>
@@ -757,12 +754,12 @@
         <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B14" t="s">
         <v>6</v>
@@ -771,12 +768,12 @@
         <v>7</v>
       </c>
       <c r="D14" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B15" t="s">
         <v>6</v>
@@ -785,12 +782,12 @@
         <v>7</v>
       </c>
       <c r="D15" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B16" t="s">
         <v>6</v>
@@ -799,12 +796,12 @@
         <v>7</v>
       </c>
       <c r="D16" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B17" t="s">
         <v>6</v>
@@ -813,12 +810,12 @@
         <v>7</v>
       </c>
       <c r="D17" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B18" t="s">
         <v>6</v>
@@ -827,12 +824,12 @@
         <v>7</v>
       </c>
       <c r="D18" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B19" t="s">
         <v>6</v>
@@ -841,12 +838,12 @@
         <v>7</v>
       </c>
       <c r="D19" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B20" t="s">
         <v>6</v>
@@ -855,12 +852,12 @@
         <v>7</v>
       </c>
       <c r="D20" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B21" t="s">
         <v>6</v>
@@ -869,12 +866,12 @@
         <v>7</v>
       </c>
       <c r="D21" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B22" t="s">
         <v>6</v>
@@ -883,12 +880,12 @@
         <v>7</v>
       </c>
       <c r="D22" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B23" t="s">
         <v>6</v>
@@ -897,12 +894,12 @@
         <v>7</v>
       </c>
       <c r="D23" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B24" t="s">
         <v>6</v>
@@ -911,12 +908,12 @@
         <v>7</v>
       </c>
       <c r="D24" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B25" t="s">
         <v>6</v>
@@ -925,12 +922,12 @@
         <v>7</v>
       </c>
       <c r="D25" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B26" t="s">
         <v>6</v>
@@ -939,12 +936,12 @@
         <v>7</v>
       </c>
       <c r="D26" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B27" t="s">
         <v>6</v>
@@ -953,12 +950,12 @@
         <v>7</v>
       </c>
       <c r="D27" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B28" t="s">
         <v>6</v>
@@ -967,12 +964,12 @@
         <v>7</v>
       </c>
       <c r="D28" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B29" t="s">
         <v>6</v>
@@ -981,12 +978,12 @@
         <v>7</v>
       </c>
       <c r="D29" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B30" t="s">
         <v>6</v>
@@ -995,12 +992,12 @@
         <v>7</v>
       </c>
       <c r="D30" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B31" t="s">
         <v>6</v>
@@ -1009,12 +1006,12 @@
         <v>7</v>
       </c>
       <c r="D31" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B32" t="s">
         <v>6</v>
@@ -1023,12 +1020,12 @@
         <v>7</v>
       </c>
       <c r="D32" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B33" t="s">
         <v>6</v>
@@ -1037,12 +1034,12 @@
         <v>7</v>
       </c>
       <c r="D33" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B34" t="s">
         <v>6</v>
@@ -1051,12 +1048,12 @@
         <v>7</v>
       </c>
       <c r="D34" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B35" t="s">
         <v>6</v>
@@ -1070,7 +1067,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B36" t="s">
         <v>6</v>
@@ -1084,7 +1081,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B37" t="s">
         <v>6</v>
@@ -1098,7 +1095,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B38" t="s">
         <v>6</v>
@@ -1112,7 +1109,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B39" t="s">
         <v>6</v>
@@ -1126,7 +1123,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B40" t="s">
         <v>6</v>
@@ -1140,7 +1137,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B41" t="s">
         <v>6</v>
@@ -1154,7 +1151,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B42" t="s">
         <v>6</v>
@@ -1168,7 +1165,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B43" t="s">
         <v>6</v>
@@ -1182,7 +1179,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B44" t="s">
         <v>6</v>
@@ -1196,7 +1193,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B45" t="s">
         <v>6</v>
@@ -1210,7 +1207,7 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B46" t="s">
         <v>6</v>
@@ -1224,7 +1221,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B47" t="s">
         <v>6</v>
@@ -1238,7 +1235,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B48" t="s">
         <v>6</v>
@@ -1252,7 +1249,7 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B49" t="s">
         <v>6</v>
@@ -1266,7 +1263,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B50" t="s">
         <v>6</v>
@@ -1280,7 +1277,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B51" t="s">
         <v>6</v>

</xml_diff>